<commit_message>
Same item numbers 1-44 on sheets 1 and 2, the lists and the equipment BOQ
- sheet 1: every item on the plan and in the equipment list carries its BOQ
  number 1-44 (list is now the 44 numbered items in BOQ order)
- sheet 2: equipment boxes carry the same numbers; power points renamed P1-P14
  so they cannot be mistaken for item numbers; HC/drain and P8/P9 moved clear
  of the dishwasher and dish sink labels
- boq-goa page, Excel, CSV and PDF use the plain numbers 1-44

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plans/kitchen-boq-goa.xlsx
+++ b/plans/kitchen-boq-goa.xlsx
@@ -540,7 +540,7 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Sl</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -610,11 +610,7 @@
       </c>
     </row>
     <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Stainless steel fabrication</t>
@@ -640,7 +636,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -695,7 +691,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -750,7 +746,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -805,7 +801,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -860,7 +856,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -915,7 +911,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -970,7 +966,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1025,7 +1021,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1080,7 +1076,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1135,7 +1131,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1190,7 +1186,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1245,7 +1241,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1300,7 +1296,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1351,7 +1347,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1400,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1449,7 +1445,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1498,7 +1494,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1568,11 +1564,7 @@
       <c r="N24" s="10" t="n"/>
     </row>
     <row r="26" ht="62" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="inlineStr"/>
       <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Cooking, cold and kitchen equipment (branded)</t>
@@ -1598,7 +1590,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1647,7 +1639,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1696,7 +1688,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1745,7 +1737,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1794,7 +1786,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1843,7 +1835,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1892,7 +1884,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1941,7 +1933,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1990,7 +1982,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -2039,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -2080,7 +2072,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -2117,7 +2109,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -2166,7 +2158,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2207,7 +2199,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2256,7 +2248,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2297,7 +2289,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>2.16</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2338,7 +2330,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2379,7 +2371,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2449,11 +2441,7 @@
       <c r="N45" s="10" t="n"/>
     </row>
     <row r="47" ht="62" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="A47" s="4" t="inlineStr"/>
       <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Hood, exhaust and ventilation</t>
@@ -2479,7 +2467,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -2534,7 +2522,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -2589,7 +2577,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -2638,7 +2626,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -2687,7 +2675,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -2736,7 +2724,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -2785,7 +2773,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -2834,7 +2822,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -2883,7 +2871,7 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>3.09</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">

</xml_diff>